<commit_message>
refactor: update data sorting logic and reconcile financial records in JSON and Excel files
</commit_message>
<xml_diff>
--- a/financial_report.xlsx
+++ b/financial_report.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -514,7 +514,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>booking 雙人房</t>
+          <t>Booking 雙人房</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
@@ -544,7 +544,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>雙人房</t>
+          <t>蔡東華雙人房</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
@@ -574,11 +574,11 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>包棟訂金/尾款</t>
+          <t>康淑汶包棟</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>15600</v>
+        <v>31200</v>
       </c>
     </row>
     <row r="5">
@@ -634,11 +634,11 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>雙人套房/升級/毛小孩</t>
+          <t>邱淑惠雙人套房/升級</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="7">
@@ -854,31 +854,31 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>expense</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>住宿</t>
+          <t>廣告</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>10位</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>9000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="15">
@@ -889,7 +889,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -904,11 +904,11 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>司領房</t>
+          <t>孟賢10位</t>
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>1000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="16">
@@ -919,7 +919,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -934,11 +934,11 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>狗狗清潔費</t>
+          <t>司領房</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>3700</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="17">
@@ -964,11 +964,11 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>春節櫻花/雅房</t>
+          <t>Booking鯉魚/狗清潔費</t>
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>8000</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="18">
@@ -979,7 +979,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -994,11 +994,11 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>兩間梅花房</t>
+          <t>趙珮妏櫻花/雅房</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>10800</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="19">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1024,11 +1024,11 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>10間房包棟</t>
+          <t>Booking兩間梅花房</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>80000</v>
+        <v>10800</v>
       </c>
     </row>
     <row r="20">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1054,11 +1054,11 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>學弟</t>
+          <t>林秀鳳包棟</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>1800</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="21">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1084,11 +1084,11 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>司領房</t>
+          <t>學弟</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>1000</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="22">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1114,11 +1114,11 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>包棟+烤肉車+紅茶</t>
+          <t>司領房</t>
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>91000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="23">
@@ -1129,26 +1129,26 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>烤肉/食材</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>食材與相關支出</t>
+          <t>陳書洋包棟+烤肉車+紅茶</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>14280</v>
+        <v>89000</v>
       </c>
     </row>
     <row r="24">
@@ -1169,16 +1169,16 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>營運</t>
+          <t>烤肉/食材</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>錦鯉</t>
+          <t>食材/雜費/飼料</t>
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>900</v>
+        <v>14280</v>
       </c>
     </row>
     <row r="25">
@@ -1199,16 +1199,16 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>烤肉/食材</t>
+          <t>營運</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>木炭</t>
+          <t>錦鯉</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>760</v>
+        <v>900</v>
       </c>
     </row>
     <row r="26">
@@ -1229,16 +1229,16 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>營運</t>
+          <t>烤肉/食材</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>飲料紙碗</t>
+          <t>木炭</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>1000</v>
+        <v>760</v>
       </c>
     </row>
     <row r="27">
@@ -1264,11 +1264,11 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>貨車加油</t>
+          <t>飲料紙碗</t>
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="28">
@@ -1294,11 +1294,11 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>魚飼料</t>
+          <t>貨車加油</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
     </row>
     <row r="29">
@@ -1319,16 +1319,16 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>早餐</t>
+          <t>營運</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>早餐合計</t>
+          <t>魚飼料</t>
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12110</v>
+        <v>250</v>
       </c>
     </row>
     <row r="30">
@@ -1349,16 +1349,16 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>房務</t>
+          <t>早餐</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>房務合計</t>
+          <t>早餐合計</t>
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>5200</v>
+        <v>12110</v>
       </c>
     </row>
     <row r="31">
@@ -1379,16 +1379,16 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>固定支出</t>
+          <t>房務</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>房租</t>
+          <t>房務合計</t>
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>70000</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="32">
@@ -1414,11 +1414,11 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>水電/稅金/網路</t>
+          <t>房租</t>
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>12864.75</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="33">
@@ -1444,112 +1444,112 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>床單清洗</t>
+          <t>水電/稅金/網路</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>7574</v>
+        <v>12864.75</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>expense</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>住宿</t>
+          <t>固定支出</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>張道宮住宿</t>
+          <t>床單清洗</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>22000</v>
+        <v>7574</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>expense</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>住宿</t>
+          <t>房務</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>林宜樑包棟</t>
+          <t>房務紅包</t>
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>31200</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>expense</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>住宿/烤肉</t>
+          <t>烤肉</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>包棟+代購烤肉食材</t>
+          <t>烤肉車</t>
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>65800</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1564,22 +1564,22 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>施正峰現收+紅茶</t>
+          <t>余小姐</t>
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>9200</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1594,112 +1594,112 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>廖小姐</t>
+          <t>董豈崧</t>
         </is>
       </c>
       <c r="F38" s="3" t="n">
-        <v>23800</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>烤肉/食材</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>烤肉支出合計</t>
+          <t>陳家揚bni</t>
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>10720</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>營運</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>雜費/用品/加油</t>
+          <t>吳家維</t>
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>4070</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>房務</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>房務合計</t>
+          <t>陳名妤2晚</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>4200</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -1709,27 +1709,27 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>早餐</t>
+          <t>廣告</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>早餐合計</t>
+          <t>Goolge</t>
         </is>
       </c>
       <c r="F42" s="3" t="n">
-        <v>8850</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1739,16 +1739,16 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>固定支出</t>
+          <t>Booking</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>房租</t>
+          <t>成交費用</t>
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>70000</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="44">
@@ -1764,21 +1764,21 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>固定支出</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>水電/稅金/網路</t>
+          <t>張道宮住宿</t>
         </is>
       </c>
       <c r="F44" s="3" t="n">
-        <v>12864.75</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="45">
@@ -1789,37 +1789,37 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>固定支出</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>床單清洗</t>
+          <t>林宜樑包棟</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>7072</v>
+        <v>31200</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -1829,27 +1829,27 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>住宿</t>
+          <t>住宿/烤肉</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>7間包棟</t>
+          <t>廖妍溱包棟2晚+烤肉</t>
         </is>
       </c>
       <c r="F46" s="3" t="n">
-        <v>28000</v>
+        <v>65800</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -1859,87 +1859,87 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>烤肉</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>烤肉</t>
+          <t>施正峰現收+紅茶</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>12000</v>
+        <v>45200</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>expense</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>住宿</t>
+          <t>烤肉/食材</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>金吉米住宿</t>
+          <t>食材/水電用品/紙碗/貨車加油</t>
         </is>
       </c>
       <c r="F48" s="3" t="n">
-        <v>7000</v>
+        <v>12282</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>expense</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>住宿/烤肉</t>
+          <t>營運</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>李雅雙住宿+代購烤肉</t>
+          <t>雜費/用品/加油</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
-        <v>15500</v>
+        <v>4070</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -1949,27 +1949,27 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>食材/營運</t>
+          <t>房務</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>4月支出合計</t>
+          <t>房務合計</t>
         </is>
       </c>
       <c r="F50" s="3" t="n">
-        <v>36543</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -1979,27 +1979,27 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>房務</t>
+          <t>早餐</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>房務費用</t>
+          <t>早餐合計</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>2500</v>
+        <v>8850</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2009,27 +2009,27 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>早餐</t>
+          <t>固定支出</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>早餐</t>
+          <t>房租</t>
         </is>
       </c>
       <c r="F52" s="3" t="n">
-        <v>2025</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2044,22 +2044,22 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>房租</t>
+          <t>水電/稅金/網路</t>
         </is>
       </c>
       <c r="F53" s="3" t="n">
-        <v>70000</v>
+        <v>12864.75</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2074,41 +2074,431 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>水電/稅金/網路</t>
+          <t>床單清洗</t>
         </is>
       </c>
       <c r="F54" s="3" t="n">
-        <v>12864.75</v>
+        <v>7072</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>收入</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>林瑞銘包棟+烤肉</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>68000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>住宿</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>許鈞翔</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>10800</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>廣告</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>住宿</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>安麗7間包棟</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>住宿</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>鍾宛蒨雙人套房</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>住宿</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>金吉米住宿</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>住宿/烤肉</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>李雅雙住宿+代購烤肉</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>15500</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>expense</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>食材/營運</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>食材/加油/濾心/貓飼料</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>36543</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>房務</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>房務費用</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>早餐</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>早餐</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>固定支出</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>房租</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>固定支出</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>水電/稅金/網路</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>12864.75</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>固定支出</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>床單清洗</t>
         </is>
       </c>
-      <c r="F55" s="3" t="n">
+      <c r="F67" s="3" t="n">
         <v>5355</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>廣告</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>18000</v>
       </c>
     </row>
   </sheetData>
@@ -2160,13 +2550,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>24500</v>
+        <v>41600</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>91070.75</v>
+        <v>109070.75</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-66570.75</v>
+        <v>-67470.75</v>
       </c>
     </row>
     <row r="3">
@@ -2176,13 +2566,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>206300</v>
+        <v>331400</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>125438.75</v>
+        <v>174938.75</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>80861.25</v>
+        <v>156461.25</v>
       </c>
     </row>
     <row r="4">
@@ -2192,13 +2582,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>152000</v>
+        <v>243000</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>117776.75</v>
+        <v>137338.75</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>34223.25</v>
+        <v>105661.25</v>
       </c>
     </row>
     <row r="5">
@@ -2208,13 +2598,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>62500</v>
+        <v>67500</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>129287.75</v>
+        <v>147287.75</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-66787.75</v>
+        <v>-79787.75</v>
       </c>
     </row>
   </sheetData>
@@ -2254,7 +2644,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>445300</v>
+        <v>683500</v>
       </c>
     </row>
     <row r="3">
@@ -2264,7 +2654,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>463574</v>
+        <v>568636</v>
       </c>
     </row>
     <row r="4">
@@ -2274,7 +2664,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>-18274</v>
+        <v>114864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: consolidate individual itemized expenses into aggregate totals for barbecue and breakfast categories
</commit_message>
<xml_diff>
--- a/financial_report.xlsx
+++ b/financial_report.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2501,6 +2501,666 @@
         <v>18000</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>住宿</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>陳俊杰 尾款</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>住宿</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Yi等3位 住宿與SUP</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>7800</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>住宿/烤肉</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>4間房、烤肉及雜項 尾款</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>22685</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>住宿</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>6大3小 尾款</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>14500</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>住宿</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>章智傑 櫻花兩人雅房</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>住宿</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>陳星妤 尾款（扣動滋卷$1000）</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>烤肉/食材</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>烤肉支出合計</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>17325</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>秋蓮 杯裝</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>秋蓮 紅茶包</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>秋蓮 包船（4/25）</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>草屯肥料</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>貓飼料</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>茶米工務車維修保養</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>金紙</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="n">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>拜拜用品</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>卡達加油</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>代買 牛排</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>1870</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>代買 鐵板麵</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>代買 滷味</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>雜費</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>代買 山東鴨頭</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>早餐</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>早餐合計</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>8165</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>房務</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>房務</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="n">
+        <v>3000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2512,7 +3172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2605,6 +3265,22 @@
       </c>
       <c r="D5" s="3" t="n">
         <v>-79787.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>62985</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>51564</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>11421</v>
       </c>
     </row>
   </sheetData>
@@ -2644,7 +3320,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>683500</v>
+        <v>746485</v>
       </c>
     </row>
     <row r="3">
@@ -2654,7 +3330,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>568636</v>
+        <v>620200</v>
       </c>
     </row>
     <row r="4">
@@ -2664,7 +3340,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>114864</v>
+        <v>126285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: normalize financial data amounts by removing redundant decimal zeros
</commit_message>
<xml_diff>
--- a/financial_report.xlsx
+++ b/financial_report.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2524,11 +2524,11 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>陳俊杰 尾款</t>
+          <t>陳俊杰</t>
         </is>
       </c>
       <c r="F69" s="3" t="n">
-        <v>14000</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="70">
@@ -2554,11 +2554,11 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Yi等3位 住宿與SUP</t>
+          <t>Yi3位住宿</t>
         </is>
       </c>
       <c r="F70" s="3" t="n">
-        <v>7800</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="71">
@@ -2584,11 +2584,11 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>4間房、烤肉及雜項 尾款</t>
+          <t>陳冠元/住宿/烤肉</t>
         </is>
       </c>
       <c r="F71" s="3" t="n">
-        <v>22685</v>
+        <v>51200</v>
       </c>
     </row>
     <row r="72">
@@ -2614,11 +2614,11 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>6大3小 尾款</t>
+          <t>劉翊炎住宿/烤肉</t>
         </is>
       </c>
       <c r="F72" s="3" t="n">
-        <v>14500</v>
+        <v>19300</v>
       </c>
     </row>
     <row r="73">
@@ -2674,11 +2674,11 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>陳星妤 尾款（扣動滋卷$1000）</t>
+          <t>陳星妤</t>
         </is>
       </c>
       <c r="F74" s="3" t="n">
-        <v>2000</v>
+        <v>5990</v>
       </c>
     </row>
     <row r="75">
@@ -2729,16 +2729,16 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>營運</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>秋蓮 杯裝</t>
+          <t>雜費合計</t>
         </is>
       </c>
       <c r="F76" s="3" t="n">
-        <v>330</v>
+        <v>22774</v>
       </c>
     </row>
     <row r="77">
@@ -2759,16 +2759,16 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>營運</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>秋蓮 紅茶包</t>
+          <t>早餐合計</t>
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>3400</v>
+        <v>8165</v>
       </c>
     </row>
     <row r="78">
@@ -2789,16 +2789,16 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>營運</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>秋蓮 包船（4/25）</t>
+          <t>房務合計</t>
         </is>
       </c>
       <c r="F78" s="3" t="n">
-        <v>10000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="79">
@@ -2819,16 +2819,16 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>固定支出</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>草屯肥料</t>
+          <t>房租</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
-        <v>300</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="80">
@@ -2849,16 +2849,16 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>固定支出</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>貓飼料</t>
+          <t>水電/稅金/網路</t>
         </is>
       </c>
       <c r="F80" s="3" t="n">
-        <v>1500</v>
+        <v>12865</v>
       </c>
     </row>
     <row r="81">
@@ -2879,16 +2879,16 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>固定支出</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>茶米工務車維修保養</t>
+          <t>床單清洗</t>
         </is>
       </c>
       <c r="F81" s="3" t="n">
-        <v>3000</v>
+        <v>7283</v>
       </c>
     </row>
     <row r="82">
@@ -2909,16 +2909,16 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>廣告</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>金紙</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="F82" s="3" t="n">
-        <v>209</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="83">
@@ -2929,26 +2929,26 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>住宿/烤肉</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>拜拜用品</t>
+          <t>李繡宇任宿/烤肉</t>
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>200</v>
+        <v>39300</v>
       </c>
     </row>
     <row r="84">
@@ -2959,26 +2959,26 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>卡達加油</t>
+          <t>龔芳琳</t>
         </is>
       </c>
       <c r="F84" s="3" t="n">
-        <v>1500</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="85">
@@ -2989,26 +2989,26 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>代買 牛排</t>
+          <t>虎哥住宿/烤肉</t>
         </is>
       </c>
       <c r="F85" s="3" t="n">
-        <v>1870</v>
+        <v>23500</v>
       </c>
     </row>
     <row r="86">
@@ -3019,26 +3019,26 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>代買 鐵板麵</t>
+          <t>果果</t>
         </is>
       </c>
       <c r="F86" s="3" t="n">
-        <v>80</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="87">
@@ -3049,26 +3049,26 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>代買 滷味</t>
+          <t>蔣思怡住宿/烤肉</t>
         </is>
       </c>
       <c r="F87" s="3" t="n">
-        <v>135</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="88">
@@ -3079,86 +3079,26 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>雜費</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>代買 山東鴨頭</t>
+          <t>劉依芳</t>
         </is>
       </c>
       <c r="F88" s="3" t="n">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>expense</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>早餐</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>早餐合計</t>
-        </is>
-      </c>
-      <c r="F89" s="3" t="n">
-        <v>8165</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>expense</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>房務</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>房務</t>
-        </is>
-      </c>
-      <c r="F90" s="3" t="n">
-        <v>3000</v>
+        <v>11500</v>
       </c>
     </row>
   </sheetData>
@@ -3274,13 +3214,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>62985</v>
+        <v>203290</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>51564</v>
+        <v>159412</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>11421</v>
+        <v>43878</v>
       </c>
     </row>
   </sheetData>
@@ -3320,7 +3260,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>746485</v>
+        <v>886790</v>
       </c>
     </row>
     <row r="3">
@@ -3330,7 +3270,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>620200</v>
+        <v>728048</v>
       </c>
     </row>
     <row r="4">
@@ -3340,7 +3280,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>126285</v>
+        <v>158742</v>
       </c>
     </row>
   </sheetData>

</xml_diff>